<commit_message>
improved automation and update to 2026
</commit_message>
<xml_diff>
--- a/Contributions_table.xlsx
+++ b/Contributions_table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lc/PycharmProjects/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F523ED88-BD44-3340-8BC2-590AB4447B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9244A3-14BF-234E-B5D8-A328E44EA3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
   </bookViews>
@@ -1092,9 +1092,6 @@
     <t>hu-etal-2024-findings</t>
   </si>
   <si>
-    <t>singh-etal-2025-global</t>
-  </si>
-  <si>
     <t>The mighty torr: A benchmark for table reasoning and robustness</t>
   </si>
   <si>
@@ -1149,9 +1146,6 @@
     <t>JML</t>
   </si>
   <si>
-    <t>wilcox2025bigger</t>
-  </si>
-  <si>
     <t>zipnn</t>
   </si>
   <si>
@@ -1234,6 +1228,12 @@
   </si>
   <si>
     <t>tam2024llm</t>
+  </si>
+  <si>
+    <t>wilcox2024bigger</t>
+  </si>
+  <si>
+    <t>singh2024global</t>
   </si>
 </sst>
 </file>
@@ -12255,7 +12255,7 @@
         <v>182</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>289</v>
@@ -15210,7 +15210,7 @@
         <v>DBLP:conf/emnlp/ChoshenVDSK23</v>
       </c>
       <c r="AJ38" t="str">
-        <f t="shared" ref="AJ38:AJ72" si="14">IF(AE38,E38,"")</f>
+        <f t="shared" ref="AJ38:AJ70" si="14">IF(AE38,E38,"")</f>
         <v/>
       </c>
     </row>
@@ -16481,7 +16481,7 @@
         <v/>
       </c>
       <c r="C55" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -17161,7 +17161,7 @@
         <v>63</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D64" t="s">
         <v>53</v>
@@ -17314,13 +17314,13 @@
         <v/>
       </c>
       <c r="C66" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D66" t="s">
         <v>163</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>339</v>
+        <v>366</v>
       </c>
       <c r="F66" t="s">
         <v>162</v>
@@ -17376,16 +17376,16 @@
         <v>1</v>
       </c>
       <c r="AG66" t="str">
-        <f t="shared" ref="AG66:AG72" si="19">IF(AF66,E66,"")</f>
-        <v>wilcox2025bigger</v>
+        <f t="shared" ref="AG66:AG71" si="19">IF(AF66,E66,"")</f>
+        <v>wilcox2024bigger</v>
       </c>
       <c r="AH66" t="str">
-        <f t="shared" ref="AH66:AH72" si="20">IF(W66,E66,"")</f>
-        <v>wilcox2025bigger</v>
+        <f t="shared" ref="AH66:AH71" si="20">IF(W66,E66,"")</f>
+        <v>wilcox2024bigger</v>
       </c>
       <c r="AI66" t="str">
-        <f t="shared" ref="AI66:AI72" si="21">IF(Y66,E66,"")</f>
-        <v>wilcox2025bigger</v>
+        <f t="shared" ref="AI66:AI71" si="21">IF(Y66,E66,"")</f>
+        <v>wilcox2024bigger</v>
       </c>
       <c r="AJ66" t="str">
         <f t="shared" si="14"/>
@@ -17456,7 +17456,7 @@
         <v>0</v>
       </c>
       <c r="AF67">
-        <f t="shared" ref="AF67:AF81" si="22">IF(SUM(T67,P67)&gt;0,1,0)</f>
+        <f t="shared" ref="AF67:AF71" si="22">IF(SUM(T67,P67)&gt;0,1,0)</f>
         <v>1</v>
       </c>
       <c r="AG67" t="str">
@@ -17486,7 +17486,7 @@
         <v/>
       </c>
       <c r="C68" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>186</v>
@@ -17875,7 +17875,7 @@
         <v/>
       </c>
       <c r="C73" t="s">
-        <v>292</v>
+        <v>185</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>275</v>
@@ -18288,7 +18288,7 @@
         <v>305</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G78">
         <v>2024</v>
@@ -18367,7 +18367,7 @@
         <v>295</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>320</v>
+        <v>367</v>
       </c>
       <c r="G79">
         <v>2024</v>
@@ -18407,15 +18407,15 @@
       </c>
       <c r="AG79" t="str">
         <f t="shared" si="25"/>
-        <v>singh-etal-2025-global</v>
+        <v>singh2024global</v>
       </c>
       <c r="AH79" t="str">
         <f t="shared" si="26"/>
-        <v>singh-etal-2025-global</v>
+        <v>singh2024global</v>
       </c>
       <c r="AI79" t="str">
         <f t="shared" si="27"/>
-        <v>singh-etal-2025-global</v>
+        <v>singh2024global</v>
       </c>
       <c r="AK79">
         <f t="shared" si="28"/>
@@ -18428,13 +18428,13 @@
         <v>79</v>
       </c>
       <c r="C80" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E80" s="12" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G80">
         <v>2025</v>
@@ -18494,10 +18494,10 @@
         <v>312</v>
       </c>
       <c r="D81" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E81" s="12" t="s">
         <v>323</v>
-      </c>
-      <c r="E81" s="12" t="s">
-        <v>324</v>
       </c>
       <c r="G81">
         <v>2025</v>
@@ -18572,10 +18572,10 @@
         <v>28</v>
       </c>
       <c r="D82" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E82" s="12" t="s">
         <v>325</v>
-      </c>
-      <c r="E82" s="12" t="s">
-        <v>326</v>
       </c>
       <c r="G82">
         <v>2025</v>
@@ -18634,16 +18634,16 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C83" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G83">
         <v>2026</v>
@@ -18706,10 +18706,10 @@
         <v>291</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G84">
         <v>2025</v>
@@ -18717,6 +18717,30 @@
       <c r="H84">
         <v>1</v>
       </c>
+      <c r="O84">
+        <v>1</v>
+      </c>
+      <c r="Q84">
+        <v>1</v>
+      </c>
+      <c r="R84">
+        <v>1</v>
+      </c>
+      <c r="S84">
+        <v>1</v>
+      </c>
+      <c r="T84">
+        <v>1</v>
+      </c>
+      <c r="U84">
+        <v>1</v>
+      </c>
+      <c r="W84">
+        <v>1</v>
+      </c>
+      <c r="Y84">
+        <v>1</v>
+      </c>
       <c r="AA84">
         <v>1</v>
       </c>
@@ -18725,19 +18749,19 @@
       </c>
       <c r="AF84">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG84" t="str">
         <f t="shared" si="25"/>
-        <v/>
+        <v>guertler2025textarena</v>
       </c>
       <c r="AH84" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>guertler2025textarena</v>
       </c>
       <c r="AI84" t="str">
         <f t="shared" si="27"/>
-        <v/>
+        <v>guertler2025textarena</v>
       </c>
       <c r="AK84">
         <f t="shared" si="28"/>
@@ -18757,10 +18781,10 @@
         <v>291</v>
       </c>
       <c r="D85" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E85" s="12" t="s">
         <v>332</v>
-      </c>
-      <c r="E85" s="12" t="s">
-        <v>333</v>
       </c>
       <c r="G85">
         <v>2025</v>
@@ -18768,6 +18792,15 @@
       <c r="H85">
         <v>1</v>
       </c>
+      <c r="P85">
+        <v>1</v>
+      </c>
+      <c r="Q85">
+        <v>1</v>
+      </c>
+      <c r="S85">
+        <v>1</v>
+      </c>
       <c r="AA85">
         <v>1</v>
       </c>
@@ -18776,11 +18809,11 @@
       </c>
       <c r="AF85">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG85" t="str">
         <f t="shared" si="25"/>
-        <v/>
+        <v>zhang2025can</v>
       </c>
       <c r="AH85" t="str">
         <f t="shared" si="26"/>
@@ -18805,18 +18838,24 @@
         <v>arxiv</v>
       </c>
       <c r="C86" t="s">
+        <v>334</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E86" s="12" t="s">
         <v>335</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="E86" s="12" t="s">
-        <v>336</v>
       </c>
       <c r="G86">
         <v>2025</v>
       </c>
       <c r="H86">
+        <v>1</v>
+      </c>
+      <c r="M86">
+        <v>1</v>
+      </c>
+      <c r="Q86">
         <v>1</v>
       </c>
       <c r="AA86">
@@ -18853,21 +18892,33 @@
       </c>
       <c r="B87" t="str" cm="1">
         <f t="array" ref="B87">_xlfn.IFS(ISBLANK(D87),"",ISBLANK(C87),"no venue",ISBLANK(E87),"no bib",ISNUMBER(SEARCH("xiv", C87)),"arxiv",SUM(I87:AA87)&lt;3,"no categories",TRUE,"")</f>
-        <v>no categories</v>
+        <v/>
       </c>
       <c r="C87" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E87" s="12" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="G87">
         <v>2025</v>
       </c>
       <c r="H87">
+        <v>1</v>
+      </c>
+      <c r="O87">
+        <v>1</v>
+      </c>
+      <c r="W87">
+        <v>1</v>
+      </c>
+      <c r="Y87">
+        <v>1</v>
+      </c>
+      <c r="Z87">
         <v>1</v>
       </c>
       <c r="AA87">
@@ -18886,11 +18937,11 @@
       </c>
       <c r="AH87" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>zipnn</v>
       </c>
       <c r="AI87" t="str">
         <f t="shared" si="27"/>
-        <v/>
+        <v>zipnn</v>
       </c>
       <c r="AK87">
         <f t="shared" si="28"/>
@@ -18904,21 +18955,27 @@
       </c>
       <c r="B88" t="str" cm="1">
         <f t="array" ref="B88">_xlfn.IFS(ISBLANK(D88),"",ISBLANK(C88),"no venue",ISBLANK(E88),"no bib",ISNUMBER(SEARCH("xiv", C88)),"arxiv",SUM(I88:AA88)&lt;3,"no categories",TRUE,"")</f>
-        <v>no categories</v>
+        <v/>
       </c>
       <c r="C88" t="s">
         <v>292</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E88" s="9" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="G88">
         <v>2025</v>
       </c>
       <c r="H88">
+        <v>1</v>
+      </c>
+      <c r="Q88">
+        <v>1</v>
+      </c>
+      <c r="S88">
         <v>1</v>
       </c>
       <c r="AA88">
@@ -18958,18 +19015,24 @@
         <v>arxiv</v>
       </c>
       <c r="C89" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="G89">
         <v>2025</v>
       </c>
       <c r="H89">
+        <v>1</v>
+      </c>
+      <c r="Q89">
+        <v>1</v>
+      </c>
+      <c r="S89">
         <v>1</v>
       </c>
       <c r="AA89">
@@ -19005,16 +19068,16 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C90" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G90">
         <v>2026</v>
@@ -19022,6 +19085,39 @@
       <c r="H90">
         <v>1</v>
       </c>
+      <c r="I90">
+        <v>1</v>
+      </c>
+      <c r="N90">
+        <v>1</v>
+      </c>
+      <c r="O90">
+        <v>1</v>
+      </c>
+      <c r="R90">
+        <v>1</v>
+      </c>
+      <c r="S90">
+        <v>1</v>
+      </c>
+      <c r="T90">
+        <v>1</v>
+      </c>
+      <c r="U90">
+        <v>1</v>
+      </c>
+      <c r="V90">
+        <v>1</v>
+      </c>
+      <c r="W90">
+        <v>1</v>
+      </c>
+      <c r="X90">
+        <v>1</v>
+      </c>
+      <c r="Y90">
+        <v>1</v>
+      </c>
       <c r="AA90">
         <v>1</v>
       </c>
@@ -19030,19 +19126,19 @@
       </c>
       <c r="AF90">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG90" t="str">
         <f t="shared" si="25"/>
-        <v/>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AH90" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AI90" t="str">
         <f t="shared" si="27"/>
-        <v/>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AK90">
         <f t="shared" si="28"/>
@@ -19059,13 +19155,13 @@
         <v>arxiv</v>
       </c>
       <c r="C91" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E91" s="12" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="G91">
         <v>2026</v>
@@ -19128,10 +19224,10 @@
         <v>310</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E92" s="12" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="G92">
         <v>2026</v>
@@ -19209,10 +19305,10 @@
         <v>no bib</v>
       </c>
       <c r="C93" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="G93">
         <v>2026</v>
@@ -19281,13 +19377,13 @@
         <v>arxiv</v>
       </c>
       <c r="C94" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E94" s="12" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="G94">
         <v>2026</v>
@@ -19350,13 +19446,13 @@
         <v>arxiv</v>
       </c>
       <c r="C95" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E95" s="12" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G95">
         <v>2026</v>
@@ -19422,13 +19518,13 @@
         <v>arxiv</v>
       </c>
       <c r="C96" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E96" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G96">
         <v>2026</v>
@@ -19482,13 +19578,13 @@
         <v>arxiv</v>
       </c>
       <c r="C97" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E97" s="12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="G97">
         <v>2026</v>
@@ -19545,7 +19641,7 @@
         <v/>
       </c>
       <c r="C98" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="G98">
         <v>2026</v>
@@ -19581,7 +19677,7 @@
         <v/>
       </c>
       <c r="C99" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="G99">
         <v>2026</v>
@@ -19598,7 +19694,7 @@
         <v/>
       </c>
       <c r="C100" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="AG100" s="8"/>
     </row>

</xml_diff>

<commit_message>
more papers in excel (uncategorized)
</commit_message>
<xml_diff>
--- a/Contributions_table.xlsx
+++ b/Contributions_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lc/PycharmProjects/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9244A3-14BF-234E-B5D8-A328E44EA3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E6D253-99C5-964F-845D-5B52E82B72C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="374">
   <si>
     <t xml:space="preserve">EMNLP (under review) </t>
   </si>
@@ -1235,12 +1235,30 @@
   <si>
     <t>singh2024global</t>
   </si>
+  <si>
+    <t>General Agent Evaluation</t>
+  </si>
+  <si>
+    <t>When AI Benchmarks Plateau: A Systematic Study of Benchmark Saturation</t>
+  </si>
+  <si>
+    <t>akhtar2026aibenchmarksplateausystematic</t>
+  </si>
+  <si>
+    <t>bandel2026generalagentevaluation</t>
+  </si>
+  <si>
+    <t>Position: Agentic Systems Should be General</t>
+  </si>
+  <si>
+    <t>bandel2026agentic</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1350,6 +1368,11 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="28"/>
+      <color rgb="FF222222"/>
+      <name val="NexusSerifWebPro"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1372,7 +1395,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
@@ -1391,6 +1414,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -19637,11 +19661,17 @@
         <v>97</v>
       </c>
       <c r="B98" t="str" cm="1">
-        <f t="array" ref="B98">_xlfn.IFS(ISBLANK(D98),"",ISBLANK(C98),"no venue",ISBLANK(E98),"no bib",ISNUMBER(SEARCH("xiv", C98)),"arxiv",SUM(I98:AA98)&lt;3,"no categories",TRUE,"")</f>
-        <v/>
+        <f t="array" ref="B98">_xlfn.IFS(ISBLANK(D99),"",ISBLANK(C98),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C98)),"arxiv",SUM(I98:AA98)&lt;3,"no categories",TRUE,"")</f>
+        <v>arxiv</v>
       </c>
       <c r="C98" t="s">
         <v>342</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E98" s="12" t="s">
+        <v>370</v>
       </c>
       <c r="G98">
         <v>2026</v>
@@ -19651,15 +19681,15 @@
         <v>0</v>
       </c>
       <c r="AG98" t="str">
-        <f t="shared" si="25"/>
+        <f>IF(AF98,#REF!,"")</f>
         <v/>
       </c>
       <c r="AH98" t="str">
-        <f t="shared" si="26"/>
+        <f>IF(W98,#REF!,"")</f>
         <v/>
       </c>
       <c r="AI98" t="str">
-        <f t="shared" si="27"/>
+        <f>IF(Y98,#REF!,"")</f>
         <v/>
       </c>
       <c r="AK98">
@@ -19673,28 +19703,43 @@
         <v>98</v>
       </c>
       <c r="B99" t="str" cm="1">
-        <f t="array" ref="B99">_xlfn.IFS(ISBLANK(D99),"",ISBLANK(C99),"no venue",ISBLANK(E99),"no bib",ISNUMBER(SEARCH("xiv", C99)),"arxiv",SUM(I99:AA99)&lt;3,"no categories",TRUE,"")</f>
-        <v/>
+        <f t="array" ref="B99">_xlfn.IFS(ISBLANK(#REF!),"",ISBLANK(C99),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C99)),"arxiv",SUM(I99:AA99)&lt;3,"no categories",TRUE,"")</f>
+        <v>arxiv</v>
       </c>
       <c r="C99" t="s">
         <v>342</v>
       </c>
+      <c r="D99" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="E99" s="12" t="s">
+        <v>371</v>
+      </c>
       <c r="G99">
         <v>2026</v>
       </c>
       <c r="AG99" s="8"/>
     </row>
-    <row r="100" spans="1:37" ht="17">
+    <row r="100" spans="1:37" ht="35">
       <c r="A100">
         <f t="shared" si="23"/>
         <v>99</v>
       </c>
       <c r="B100" t="str" cm="1">
         <f t="array" ref="B100">_xlfn.IFS(ISBLANK(D100),"",ISBLANK(C100),"no venue",ISBLANK(E100),"no bib",ISNUMBER(SEARCH("xiv", C100)),"arxiv",SUM(I100:AA100)&lt;3,"no categories",TRUE,"")</f>
-        <v/>
+        <v>arxiv</v>
       </c>
       <c r="C100" t="s">
         <v>342</v>
+      </c>
+      <c r="D100" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="E100" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="G100">
+        <v>2026</v>
       </c>
       <c r="AG100" s="8"/>
     </row>
@@ -20305,6 +20350,8 @@
     <hyperlink ref="D95" r:id="rId49" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:B3FOqHPlNUQC" xr:uid="{4655ADB8-FEB9-6148-99F7-03736D7EB3B9}"/>
     <hyperlink ref="D96" r:id="rId50" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:sSrBHYA8nusC" xr:uid="{94FB61E5-5F04-5645-A99F-119289B9E81D}"/>
     <hyperlink ref="D97" r:id="rId51" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:5Ul4iDaHHb8C" xr:uid="{AC018292-7C41-B947-89FB-2E8002093149}"/>
+    <hyperlink ref="D99" r:id="rId52" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:eflP2zaiRacC" xr:uid="{60D0073E-0896-9C4A-A723-621180E109EC}"/>
+    <hyperlink ref="D98" r:id="rId53" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:VOx2b1Wkg3QC" xr:uid="{1B316D5B-F142-5C4C-8594-5D8D28179250}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
update more papers, fix issues with previous papers
</commit_message>
<xml_diff>
--- a/Contributions_table.xlsx
+++ b/Contributions_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lc/PycharmProjects/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E6D253-99C5-964F-845D-5B52E82B72C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D359E718-0965-6D4D-AF45-A054575C6F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="376">
   <si>
     <t xml:space="preserve">EMNLP (under review) </t>
   </si>
@@ -225,9 +225,6 @@
   </si>
   <si>
     <t xml:space="preserve"> Benchmark Agreement Testing Done Right: A Guide for LLM Benchmark Evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Learning from Naturally Occurring Feedback</t>
   </si>
   <si>
     <t xml:space="preserve"> NumeroLogic: Number Encoding for Enhanced LLMs' Numerical Reasoning</t>
@@ -1000,9 +997,6 @@
     <t>ICLR</t>
   </si>
   <si>
-    <t>Review</t>
-  </si>
-  <si>
     <t>Workshop-paper</t>
   </si>
   <si>
@@ -1252,6 +1246,18 @@
   </si>
   <si>
     <t>bandel2026agentic</t>
+  </si>
+  <si>
+    <t>Review, Survey and Position</t>
+  </si>
+  <si>
+    <t>Naturally occurring feedback is common, extractable and useful</t>
+  </si>
+  <si>
+    <t>fandina2025safesafetymetricautomatic</t>
+  </si>
+  <si>
+    <t>How Safe is Your Safety Metric? Automatic Concatenation Tests for Metric Reliability</t>
   </si>
 </sst>
 </file>
@@ -12260,7 +12266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92277768-849A-7540-AC05-5E1BE041CC8E}">
-  <dimension ref="A1:AK138"/>
+  <dimension ref="A1:AK139"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="4" max="4" width="29.5" customWidth="1"/>
@@ -12276,115 +12282,115 @@
   <sheetData>
     <row r="1" spans="1:37" s="15" customFormat="1" ht="51">
       <c r="A1" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C1" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>287</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="Q1" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="R1" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="S1" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="T1" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="U1" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="V1" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="W1" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="X1" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="Y1" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="Z1" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA1" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="AB1" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="AC1" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="AD1" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="AE1" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="AF1" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="AG1" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="AH1" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="AI1" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="AJ1" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="AK1" s="15" t="s">
         <v>289</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>247</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>259</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>288</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="K1" s="15" t="s">
-        <v>284</v>
-      </c>
-      <c r="L1" s="15" t="s">
-        <v>283</v>
-      </c>
-      <c r="M1" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="N1" s="15" t="s">
-        <v>285</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>261</v>
-      </c>
-      <c r="P1" s="15" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q1" s="15" t="s">
-        <v>260</v>
-      </c>
-      <c r="R1" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="S1" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="T1" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="U1" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="V1" s="15" t="s">
-        <v>262</v>
-      </c>
-      <c r="W1" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="X1" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="Y1" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="Z1" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="AA1" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="AB1" s="15" t="s">
-        <v>294</v>
-      </c>
-      <c r="AC1" s="15" t="s">
-        <v>293</v>
-      </c>
-      <c r="AD1" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="AE1" s="15" t="s">
-        <v>257</v>
-      </c>
-      <c r="AF1" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="AG1" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="AH1" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="AI1" s="15" t="s">
-        <v>250</v>
-      </c>
-      <c r="AJ1" s="15" t="s">
-        <v>257</v>
-      </c>
-      <c r="AK1" s="15" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="2" spans="1:37">
@@ -12402,10 +12408,10 @@
         <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G2">
         <v>2018</v>
@@ -12461,16 +12467,16 @@
         <v/>
       </c>
       <c r="C3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>127</v>
-      </c>
       <c r="E3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G3">
         <v>2018</v>
@@ -12539,13 +12545,13 @@
         <v>46</v>
       </c>
       <c r="D4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F4" t="s">
         <v>124</v>
-      </c>
-      <c r="E4" t="s">
-        <v>206</v>
-      </c>
-      <c r="F4" t="s">
-        <v>125</v>
       </c>
       <c r="G4">
         <v>2018</v>
@@ -12612,13 +12618,13 @@
         <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G5">
         <v>2018</v>
@@ -12699,13 +12705,13 @@
         <v>44</v>
       </c>
       <c r="D6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G6">
         <v>2018</v>
@@ -12774,13 +12780,13 @@
         <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7">
         <v>2019</v>
@@ -12864,13 +12870,13 @@
         <v>42</v>
       </c>
       <c r="D8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" t="s">
+        <v>233</v>
+      </c>
+      <c r="F8" t="s">
         <v>118</v>
-      </c>
-      <c r="E8" t="s">
-        <v>234</v>
-      </c>
-      <c r="F8" t="s">
-        <v>119</v>
       </c>
       <c r="G8">
         <v>2019</v>
@@ -12934,13 +12940,13 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E9" t="s">
+        <v>232</v>
+      </c>
+      <c r="F9" t="s">
         <v>116</v>
-      </c>
-      <c r="E9" t="s">
-        <v>233</v>
-      </c>
-      <c r="F9" t="s">
-        <v>117</v>
       </c>
       <c r="G9">
         <v>2019</v>
@@ -13009,13 +13015,13 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" t="s">
+        <v>231</v>
+      </c>
+      <c r="F10" t="s">
         <v>114</v>
-      </c>
-      <c r="E10" t="s">
-        <v>232</v>
-      </c>
-      <c r="F10" t="s">
-        <v>115</v>
       </c>
       <c r="G10">
         <v>2019</v>
@@ -13097,13 +13103,13 @@
         <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G11">
         <v>2019</v>
@@ -13187,13 +13193,13 @@
         <v>38</v>
       </c>
       <c r="D12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E12" t="s">
+        <v>229</v>
+      </c>
+      <c r="F12" t="s">
         <v>110</v>
-      </c>
-      <c r="E12" t="s">
-        <v>230</v>
-      </c>
-      <c r="F12" t="s">
-        <v>111</v>
       </c>
       <c r="G12">
         <v>2020</v>
@@ -13266,13 +13272,13 @@
         <v>37</v>
       </c>
       <c r="D13" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" t="s">
+        <v>228</v>
+      </c>
+      <c r="F13" t="s">
         <v>146</v>
-      </c>
-      <c r="E13" t="s">
-        <v>229</v>
-      </c>
-      <c r="F13" t="s">
-        <v>147</v>
       </c>
       <c r="G13">
         <v>2020</v>
@@ -13343,13 +13349,13 @@
         <v>36</v>
       </c>
       <c r="D14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E14" t="s">
+        <v>204</v>
+      </c>
+      <c r="F14" t="s">
         <v>144</v>
-      </c>
-      <c r="E14" t="s">
-        <v>205</v>
-      </c>
-      <c r="F14" t="s">
-        <v>145</v>
       </c>
       <c r="G14">
         <v>2020</v>
@@ -13409,13 +13415,13 @@
         <v>35</v>
       </c>
       <c r="D15" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" t="s">
+        <v>227</v>
+      </c>
+      <c r="F15" t="s">
         <v>142</v>
-      </c>
-      <c r="E15" t="s">
-        <v>228</v>
-      </c>
-      <c r="F15" t="s">
-        <v>143</v>
       </c>
       <c r="G15">
         <v>2020</v>
@@ -13486,13 +13492,13 @@
         <v>34</v>
       </c>
       <c r="D16" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" t="s">
+        <v>226</v>
+      </c>
+      <c r="F16" t="s">
         <v>140</v>
-      </c>
-      <c r="E16" t="s">
-        <v>227</v>
-      </c>
-      <c r="F16" t="s">
-        <v>141</v>
       </c>
       <c r="G16">
         <v>2020</v>
@@ -13572,13 +13578,13 @@
         <v>33</v>
       </c>
       <c r="D17" t="s">
+        <v>137</v>
+      </c>
+      <c r="E17" t="s">
+        <v>203</v>
+      </c>
+      <c r="F17" t="s">
         <v>138</v>
-      </c>
-      <c r="E17" t="s">
-        <v>204</v>
-      </c>
-      <c r="F17" t="s">
-        <v>139</v>
       </c>
       <c r="G17">
         <v>2020</v>
@@ -13650,13 +13656,13 @@
         <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G18" s="4">
         <v>2021</v>
@@ -13729,13 +13735,13 @@
         <v>31</v>
       </c>
       <c r="D19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" t="s">
+        <v>225</v>
+      </c>
+      <c r="F19" t="s">
         <v>93</v>
-      </c>
-      <c r="E19" t="s">
-        <v>226</v>
-      </c>
-      <c r="F19" t="s">
-        <v>94</v>
       </c>
       <c r="G19" s="4">
         <v>2021</v>
@@ -13797,13 +13803,13 @@
         <v>30</v>
       </c>
       <c r="D20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" t="s">
+        <v>201</v>
+      </c>
+      <c r="F20" t="s">
         <v>91</v>
-      </c>
-      <c r="E20" t="s">
-        <v>202</v>
-      </c>
-      <c r="F20" t="s">
-        <v>92</v>
       </c>
       <c r="G20" s="4">
         <v>2021</v>
@@ -13877,13 +13883,13 @@
         <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E21" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G21" s="4">
         <v>2021</v>
@@ -13948,13 +13954,13 @@
         <v>28</v>
       </c>
       <c r="D22" t="s">
+        <v>88</v>
+      </c>
+      <c r="E22" t="s">
+        <v>200</v>
+      </c>
+      <c r="F22" t="s">
         <v>89</v>
-      </c>
-      <c r="E22" t="s">
-        <v>201</v>
-      </c>
-      <c r="F22" t="s">
-        <v>90</v>
       </c>
       <c r="G22">
         <v>2022</v>
@@ -14013,13 +14019,13 @@
         <v>28</v>
       </c>
       <c r="D23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" t="s">
+        <v>199</v>
+      </c>
+      <c r="F23" t="s">
         <v>87</v>
-      </c>
-      <c r="E23" t="s">
-        <v>200</v>
-      </c>
-      <c r="F23" t="s">
-        <v>88</v>
       </c>
       <c r="G23">
         <v>2022</v>
@@ -14081,13 +14087,13 @@
         <v>27</v>
       </c>
       <c r="D24" t="s">
+        <v>84</v>
+      </c>
+      <c r="E24" t="s">
+        <v>239</v>
+      </c>
+      <c r="F24" t="s">
         <v>85</v>
-      </c>
-      <c r="E24" t="s">
-        <v>240</v>
-      </c>
-      <c r="F24" t="s">
-        <v>86</v>
       </c>
       <c r="G24">
         <v>2022</v>
@@ -14159,13 +14165,13 @@
         <v>26</v>
       </c>
       <c r="D25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G25">
         <v>2022</v>
@@ -14239,13 +14245,13 @@
         <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E26" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G26">
         <v>2023</v>
@@ -14315,13 +14321,13 @@
         <v>24</v>
       </c>
       <c r="D27" t="s">
+        <v>82</v>
+      </c>
+      <c r="E27" t="s">
+        <v>198</v>
+      </c>
+      <c r="F27" t="s">
         <v>83</v>
-      </c>
-      <c r="E27" t="s">
-        <v>199</v>
-      </c>
-      <c r="F27" t="s">
-        <v>84</v>
       </c>
       <c r="G27">
         <v>2023</v>
@@ -14402,13 +14408,13 @@
         <v>23</v>
       </c>
       <c r="D28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>221</v>
+      </c>
+      <c r="F28" t="s">
         <v>81</v>
-      </c>
-      <c r="E28" t="s">
-        <v>222</v>
-      </c>
-      <c r="F28" t="s">
-        <v>82</v>
       </c>
       <c r="G28">
         <v>2023</v>
@@ -14473,13 +14479,13 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G29">
         <v>2023</v>
@@ -14542,13 +14548,13 @@
         <v>18</v>
       </c>
       <c r="D30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E30" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F30" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G30">
         <v>2023</v>
@@ -14625,13 +14631,13 @@
         <v>21</v>
       </c>
       <c r="D31" t="s">
+        <v>77</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="F31" t="s">
         <v>78</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="F31" t="s">
-        <v>79</v>
       </c>
       <c r="G31">
         <v>2023</v>
@@ -14696,13 +14702,13 @@
         <v>20</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G32">
         <v>2023</v>
@@ -14776,13 +14782,13 @@
         <v>19</v>
       </c>
       <c r="D33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" t="s">
+        <v>197</v>
+      </c>
+      <c r="F33" t="s">
         <v>75</v>
-      </c>
-      <c r="E33" t="s">
-        <v>198</v>
-      </c>
-      <c r="F33" t="s">
-        <v>76</v>
       </c>
       <c r="G33">
         <v>2023</v>
@@ -14845,13 +14851,13 @@
         <v>18</v>
       </c>
       <c r="D34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G34">
         <v>2023</v>
@@ -14916,13 +14922,13 @@
         <v>17</v>
       </c>
       <c r="D35" t="s">
+        <v>71</v>
+      </c>
+      <c r="E35" t="s">
+        <v>216</v>
+      </c>
+      <c r="F35" t="s">
         <v>72</v>
-      </c>
-      <c r="E35" t="s">
-        <v>217</v>
-      </c>
-      <c r="F35" t="s">
-        <v>73</v>
       </c>
       <c r="G35">
         <v>2023</v>
@@ -14987,13 +14993,13 @@
         <v>16</v>
       </c>
       <c r="D36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E36" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G36">
         <v>2023</v>
@@ -15063,16 +15069,16 @@
         <v/>
       </c>
       <c r="C37" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D37" t="s">
         <v>268</v>
       </c>
-      <c r="D37" t="s">
-        <v>269</v>
-      </c>
       <c r="E37" t="s">
+        <v>264</v>
+      </c>
+      <c r="F37" t="s">
         <v>265</v>
-      </c>
-      <c r="F37" t="s">
-        <v>266</v>
       </c>
       <c r="G37">
         <v>2023</v>
@@ -15160,13 +15166,13 @@
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E38" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G38">
         <v>2023</v>
@@ -15251,13 +15257,13 @@
         <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E39" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G39">
         <v>2023</v>
@@ -15316,13 +15322,13 @@
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E40" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G40">
         <v>2023</v>
@@ -15391,13 +15397,13 @@
         <v>14</v>
       </c>
       <c r="D41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E41" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F41" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G41">
         <v>2023</v>
@@ -15469,13 +15475,13 @@
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E42" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F42" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G42">
         <v>2023</v>
@@ -15543,13 +15549,13 @@
         <v>12</v>
       </c>
       <c r="D43" t="s">
+        <v>66</v>
+      </c>
+      <c r="E43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F43" t="s">
         <v>67</v>
-      </c>
-      <c r="E43" t="s">
-        <v>196</v>
-      </c>
-      <c r="F43" t="s">
-        <v>68</v>
       </c>
       <c r="G43">
         <v>2024</v>
@@ -15627,16 +15633,16 @@
         <v/>
       </c>
       <c r="C44" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D44" t="s">
         <v>176</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
+        <v>194</v>
+      </c>
+      <c r="F44" t="s">
         <v>177</v>
-      </c>
-      <c r="E44" t="s">
-        <v>195</v>
-      </c>
-      <c r="F44" t="s">
-        <v>178</v>
       </c>
       <c r="G44">
         <v>2024</v>
@@ -15699,16 +15705,16 @@
         <v/>
       </c>
       <c r="C45" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D45" t="s">
+        <v>272</v>
+      </c>
+      <c r="E45" t="s">
+        <v>271</v>
+      </c>
+      <c r="F45" t="s">
         <v>273</v>
-      </c>
-      <c r="E45" t="s">
-        <v>272</v>
-      </c>
-      <c r="F45" t="s">
-        <v>274</v>
       </c>
       <c r="G45">
         <v>2024</v>
@@ -15780,13 +15786,13 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F46" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G46">
         <v>2024</v>
@@ -15855,13 +15861,13 @@
         <v>10</v>
       </c>
       <c r="D47" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" t="s">
+        <v>212</v>
+      </c>
+      <c r="F47" t="s">
         <v>64</v>
-      </c>
-      <c r="E47" t="s">
-        <v>213</v>
-      </c>
-      <c r="F47" t="s">
-        <v>65</v>
       </c>
       <c r="G47">
         <v>2024</v>
@@ -15926,13 +15932,13 @@
         <v>9</v>
       </c>
       <c r="D48" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E48" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F48" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G48">
         <v>2024</v>
@@ -16027,13 +16033,13 @@
         <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E49" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G49">
         <v>2024</v>
@@ -16104,13 +16110,13 @@
         <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E50" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F50" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G50">
         <v>2024</v>
@@ -16178,13 +16184,13 @@
         <v>7</v>
       </c>
       <c r="D51" t="s">
+        <v>61</v>
+      </c>
+      <c r="E51" t="s">
+        <v>209</v>
+      </c>
+      <c r="F51" t="s">
         <v>62</v>
-      </c>
-      <c r="E51" t="s">
-        <v>210</v>
-      </c>
-      <c r="F51" t="s">
-        <v>63</v>
       </c>
       <c r="G51">
         <v>2024</v>
@@ -16259,13 +16265,13 @@
         <v>6</v>
       </c>
       <c r="D52" t="s">
+        <v>59</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="F52" t="s">
         <v>60</v>
-      </c>
-      <c r="E52" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="F52" t="s">
-        <v>61</v>
       </c>
       <c r="G52">
         <v>2024</v>
@@ -16346,13 +16352,13 @@
         <v>5</v>
       </c>
       <c r="D53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E53" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F53" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G53">
         <v>2024</v>
@@ -16427,13 +16433,13 @@
         <v>4</v>
       </c>
       <c r="D54" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E54" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F54" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G54">
         <v>2024</v>
@@ -16505,16 +16511,16 @@
         <v/>
       </c>
       <c r="C55" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D55" t="s">
+        <v>56</v>
+      </c>
+      <c r="E55" t="s">
+        <v>243</v>
+      </c>
+      <c r="F55" t="s">
         <v>57</v>
-      </c>
-      <c r="E55" t="s">
-        <v>244</v>
-      </c>
-      <c r="F55" t="s">
-        <v>58</v>
       </c>
       <c r="G55">
         <v>2024</v>
@@ -16582,13 +16588,13 @@
         <v/>
       </c>
       <c r="C56" s="2" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E56" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F56" t="s">
         <v>3</v>
@@ -16663,16 +16669,16 @@
         <v/>
       </c>
       <c r="C57" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D57" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="F57" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G57">
         <v>2024</v>
@@ -16741,16 +16747,16 @@
         <v/>
       </c>
       <c r="C58" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D58" t="s">
+        <v>54</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="F58" t="s">
         <v>55</v>
-      </c>
-      <c r="E58" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="F58" t="s">
-        <v>56</v>
       </c>
       <c r="G58">
         <v>2024</v>
@@ -16812,13 +16818,13 @@
         <v>1</v>
       </c>
       <c r="D59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E59" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F59" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G59">
         <v>2024</v>
@@ -16884,16 +16890,16 @@
         <v/>
       </c>
       <c r="C60" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G60">
         <v>2024</v>
@@ -16959,7 +16965,7 @@
         <v>49</v>
       </c>
       <c r="E61" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F61" t="s">
         <v>2</v>
@@ -17022,16 +17028,16 @@
         <v/>
       </c>
       <c r="C62" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D62" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="F62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G62">
         <v>2024</v>
@@ -17110,14 +17116,14 @@
       <c r="C63" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D63" t="s">
-        <v>54</v>
+      <c r="D63" s="2" t="s">
+        <v>373</v>
       </c>
       <c r="E63" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F63" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G63">
         <v>2024</v>
@@ -17185,16 +17191,16 @@
         <v>63</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D64" t="s">
         <v>53</v>
       </c>
       <c r="E64" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F64" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G64">
         <v>2024</v>
@@ -17260,16 +17266,16 @@
         <v/>
       </c>
       <c r="C65" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D65" t="s">
         <v>52</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="F65" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G65">
         <v>2024</v>
@@ -17338,16 +17344,16 @@
         <v/>
       </c>
       <c r="C66" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D66" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F66" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G66">
         <v>2024</v>
@@ -17436,7 +17442,7 @@
         <v>50</v>
       </c>
       <c r="E67" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F67" t="s">
         <v>51</v>
@@ -17502,7 +17508,7 @@
     </row>
     <row r="68" spans="1:37">
       <c r="A68">
-        <f t="shared" ref="A68:A127" si="23">1+A67</f>
+        <f t="shared" ref="A68:A128" si="23">1+A67</f>
         <v>67</v>
       </c>
       <c r="B68" t="str" cm="1">
@@ -17510,16 +17516,16 @@
         <v/>
       </c>
       <c r="C68" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D68" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E68" t="s">
+        <v>187</v>
+      </c>
+      <c r="F68" t="s">
         <v>186</v>
-      </c>
-      <c r="E68" t="s">
-        <v>188</v>
-      </c>
-      <c r="F68" t="s">
-        <v>187</v>
       </c>
       <c r="G68">
         <v>2024</v>
@@ -17544,6 +17550,9 @@
         <v>1</v>
       </c>
       <c r="AA68">
+        <v>1</v>
+      </c>
+      <c r="AC68">
         <v>1</v>
       </c>
       <c r="AD68">
@@ -17584,16 +17593,16 @@
         <v/>
       </c>
       <c r="C69" t="s">
+        <v>250</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="E69" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F69" s="10" t="s">
         <v>252</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="F69" s="10" t="s">
-        <v>253</v>
       </c>
       <c r="G69">
         <v>2024</v>
@@ -17652,16 +17661,16 @@
         <v/>
       </c>
       <c r="C70" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D70" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="F70" s="10" t="s">
         <v>255</v>
-      </c>
-      <c r="E70" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="F70" s="10" t="s">
-        <v>256</v>
       </c>
       <c r="G70">
         <v>2024</v>
@@ -17670,6 +17679,9 @@
         <v>1</v>
       </c>
       <c r="K70">
+        <v>1</v>
+      </c>
+      <c r="N70">
         <v>1</v>
       </c>
       <c r="P70">
@@ -17723,16 +17735,16 @@
         <v/>
       </c>
       <c r="C71" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D71" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E71" s="12" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F71" s="10" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="G71">
         <v>2024</v>
@@ -17817,16 +17829,16 @@
         <v/>
       </c>
       <c r="C72" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E72" t="s">
+        <v>269</v>
+      </c>
+      <c r="F72" s="10" t="s">
         <v>270</v>
-      </c>
-      <c r="F72" s="10" t="s">
-        <v>271</v>
       </c>
       <c r="G72">
         <v>2024</v>
@@ -17869,7 +17881,7 @@
         <v>0</v>
       </c>
       <c r="AF72">
-        <f t="shared" ref="AF72:AF98" si="24">IF(SUM(T72,P72)&gt;0,1,0)</f>
+        <f t="shared" ref="AF72:AF99" si="24">IF(SUM(T72,P72)&gt;0,1,0)</f>
         <v>1</v>
       </c>
       <c r="AG72" t="str">
@@ -17885,7 +17897,7 @@
         <v>knots</v>
       </c>
       <c r="AK72">
-        <f t="shared" ref="AK72:AK98" si="28">IF(Z72+T72&gt;1,1,0)</f>
+        <f t="shared" ref="AK72:AK101" si="28">IF(Z72+T72&gt;1,1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -17899,16 +17911,16 @@
         <v/>
       </c>
       <c r="C73" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D73" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E73" t="s">
+        <v>281</v>
+      </c>
+      <c r="F73" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="E73" t="s">
-        <v>282</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>276</v>
       </c>
       <c r="G73">
         <v>2024</v>
@@ -17987,16 +17999,16 @@
         <v/>
       </c>
       <c r="C74" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D74" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E74" t="s">
+        <v>278</v>
+      </c>
+      <c r="F74" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="E74" t="s">
-        <v>279</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>278</v>
       </c>
       <c r="G74">
         <v>2024</v>
@@ -18080,16 +18092,16 @@
         <v>74</v>
       </c>
       <c r="C75" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D75" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="E75" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="F75" s="5" t="s">
         <v>297</v>
-      </c>
-      <c r="E75" s="12" t="s">
-        <v>298</v>
-      </c>
-      <c r="F75" s="5" t="s">
-        <v>299</v>
       </c>
       <c r="G75">
         <v>2024</v>
@@ -18160,16 +18172,16 @@
         <v/>
       </c>
       <c r="C76" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D76" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="F76" s="5" t="s">
         <v>280</v>
-      </c>
-      <c r="E76" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>281</v>
       </c>
       <c r="G76">
         <v>2024</v>
@@ -18224,13 +18236,13 @@
         <v/>
       </c>
       <c r="C77" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D77" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E77" s="12" t="s">
         <v>317</v>
-      </c>
-      <c r="E77" s="12" t="s">
-        <v>319</v>
       </c>
       <c r="G77">
         <v>2024</v>
@@ -18306,13 +18318,13 @@
         <v/>
       </c>
       <c r="C78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="G78">
         <v>2024</v>
@@ -18385,13 +18397,13 @@
         <v/>
       </c>
       <c r="C79" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G79">
         <v>2024</v>
@@ -18452,13 +18464,13 @@
         <v>79</v>
       </c>
       <c r="C80" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E80" s="12" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="G80">
         <v>2025</v>
@@ -18515,13 +18527,13 @@
         <v/>
       </c>
       <c r="C81" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E81" s="12" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G81">
         <v>2025</v>
@@ -18596,10 +18608,10 @@
         <v>28</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E82" s="12" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="G82">
         <v>2025</v>
@@ -18658,16 +18670,16 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C83" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="G83">
         <v>2026</v>
@@ -18727,13 +18739,13 @@
         <v>arxiv</v>
       </c>
       <c r="C84" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D84" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="E84" s="12" t="s">
         <v>327</v>
-      </c>
-      <c r="E84" s="12" t="s">
-        <v>329</v>
       </c>
       <c r="G84">
         <v>2025</v>
@@ -18802,13 +18814,13 @@
         <v>arxiv</v>
       </c>
       <c r="C85" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E85" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G85">
         <v>2025</v>
@@ -18862,13 +18874,13 @@
         <v>arxiv</v>
       </c>
       <c r="C86" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D86" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E86" s="12" t="s">
         <v>333</v>
-      </c>
-      <c r="E86" s="12" t="s">
-        <v>335</v>
       </c>
       <c r="G86">
         <v>2025</v>
@@ -18919,13 +18931,13 @@
         <v/>
       </c>
       <c r="C87" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D87" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E87" s="12" t="s">
         <v>336</v>
-      </c>
-      <c r="E87" s="12" t="s">
-        <v>338</v>
       </c>
       <c r="G87">
         <v>2025</v>
@@ -18982,13 +18994,13 @@
         <v/>
       </c>
       <c r="C88" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E88" s="9" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G88">
         <v>2025</v>
@@ -19039,13 +19051,13 @@
         <v>arxiv</v>
       </c>
       <c r="C89" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="G89">
         <v>2025</v>
@@ -19091,57 +19103,28 @@
         <f t="shared" si="23"/>
         <v>89</v>
       </c>
-      <c r="B90" t="s">
-        <v>349</v>
+      <c r="B90" t="str" cm="1">
+        <f t="array" ref="B90">_xlfn.IFS(ISBLANK(D90),"",ISBLANK(C90),"no venue",ISBLANK(E90),"no bib",ISNUMBER(SEARCH("xiv", C90)),"arxiv",SUM(I90:AA90)&lt;3,"no categories",TRUE,"")</f>
+        <v>arxiv</v>
       </c>
       <c r="C90" t="s">
-        <v>345</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>348</v>
+        <v>290</v>
+      </c>
+      <c r="D90" s="9" t="s">
+        <v>375</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>352</v>
+        <v>374</v>
       </c>
       <c r="G90">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="H90">
         <v>1</v>
       </c>
-      <c r="I90">
-        <v>1</v>
-      </c>
-      <c r="N90">
-        <v>1</v>
-      </c>
-      <c r="O90">
-        <v>1</v>
-      </c>
-      <c r="R90">
-        <v>1</v>
-      </c>
-      <c r="S90">
-        <v>1</v>
-      </c>
       <c r="T90">
         <v>1</v>
       </c>
-      <c r="U90">
-        <v>1</v>
-      </c>
-      <c r="V90">
-        <v>1</v>
-      </c>
-      <c r="W90">
-        <v>1</v>
-      </c>
-      <c r="X90">
-        <v>1</v>
-      </c>
-      <c r="Y90">
-        <v>1</v>
-      </c>
       <c r="AA90">
         <v>1</v>
       </c>
@@ -19149,23 +19132,23 @@
         <v>1</v>
       </c>
       <c r="AF90">
-        <f t="shared" si="24"/>
+        <f t="shared" ref="AF90" si="30">IF(SUM(T90,P90)&gt;0,1,0)</f>
         <v>1</v>
       </c>
       <c r="AG90" t="str">
-        <f t="shared" si="25"/>
-        <v>jumelet2025babybabellm</v>
+        <f t="shared" ref="AG90" si="31">IF(AF90,E90,"")</f>
+        <v>fandina2025safesafetymetricautomatic</v>
       </c>
       <c r="AH90" t="str">
-        <f t="shared" si="26"/>
-        <v>jumelet2025babybabellm</v>
+        <f t="shared" ref="AH90" si="32">IF(W90,E90,"")</f>
+        <v/>
       </c>
       <c r="AI90" t="str">
-        <f t="shared" si="27"/>
-        <v>jumelet2025babybabellm</v>
+        <f t="shared" ref="AI90" si="33">IF(Y90,E90,"")</f>
+        <v/>
       </c>
       <c r="AK90">
-        <f t="shared" si="28"/>
+        <f t="shared" ref="AK90" si="34">IF(Z90+T90&gt;1,1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -19174,18 +19157,17 @@
         <f t="shared" si="23"/>
         <v>90</v>
       </c>
-      <c r="B91" t="str" cm="1">
-        <f t="array" ref="B91">_xlfn.IFS(ISBLANK(D91),"",ISBLANK(C91),"no venue",ISBLANK(E91),"no bib",ISNUMBER(SEARCH("xiv", C91)),"arxiv",SUM(I91:AA91)&lt;3,"no categories",TRUE,"")</f>
-        <v>arxiv</v>
+      <c r="B91" t="s">
+        <v>347</v>
       </c>
       <c r="C91" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D91" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="E91" s="12" t="s">
         <v>350</v>
-      </c>
-      <c r="E91" s="12" t="s">
-        <v>351</v>
       </c>
       <c r="G91">
         <v>2026</v>
@@ -19193,6 +19175,9 @@
       <c r="H91">
         <v>1</v>
       </c>
+      <c r="I91">
+        <v>1</v>
+      </c>
       <c r="N91">
         <v>1</v>
       </c>
@@ -19202,7 +19187,22 @@
       <c r="R91">
         <v>1</v>
       </c>
+      <c r="S91">
+        <v>1</v>
+      </c>
+      <c r="T91">
+        <v>1</v>
+      </c>
       <c r="U91">
+        <v>1</v>
+      </c>
+      <c r="V91">
+        <v>1</v>
+      </c>
+      <c r="W91">
+        <v>1</v>
+      </c>
+      <c r="X91">
         <v>1</v>
       </c>
       <c r="Y91">
@@ -19216,19 +19216,19 @@
       </c>
       <c r="AF91">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG91" t="str">
         <f t="shared" si="25"/>
-        <v/>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AH91" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AI91" t="str">
         <f t="shared" si="27"/>
-        <v>chang2025globalpiqaevaluatingphysical</v>
+        <v>jumelet2025babybabellm</v>
       </c>
       <c r="AK91">
         <f t="shared" si="28"/>
@@ -19242,16 +19242,16 @@
       </c>
       <c r="B92" t="str" cm="1">
         <f t="array" ref="B92">_xlfn.IFS(ISBLANK(D92),"",ISBLANK(C92),"no venue",ISBLANK(E92),"no bib",ISNUMBER(SEARCH("xiv", C92)),"arxiv",SUM(I92:AA92)&lt;3,"no categories",TRUE,"")</f>
-        <v/>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>310</v>
+        <v>arxiv</v>
+      </c>
+      <c r="C92" t="s">
+        <v>340</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="E92" s="12" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="G92">
         <v>2026</v>
@@ -19259,40 +19259,22 @@
       <c r="H92">
         <v>1</v>
       </c>
-      <c r="I92">
-        <v>1</v>
-      </c>
       <c r="N92">
         <v>1</v>
       </c>
       <c r="O92">
         <v>1</v>
       </c>
-      <c r="Q92">
-        <v>1</v>
-      </c>
       <c r="R92">
         <v>1</v>
       </c>
-      <c r="S92">
-        <v>1</v>
-      </c>
-      <c r="T92">
-        <v>1</v>
-      </c>
       <c r="U92">
         <v>1</v>
       </c>
-      <c r="V92">
-        <v>1</v>
-      </c>
-      <c r="Z92">
+      <c r="Y92">
         <v>1</v>
       </c>
       <c r="AA92">
-        <v>1</v>
-      </c>
-      <c r="AB92">
         <v>1</v>
       </c>
       <c r="AD92">
@@ -19300,11 +19282,11 @@
       </c>
       <c r="AF92">
         <f t="shared" si="24"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG92" t="str">
         <f t="shared" si="25"/>
-        <v>charpentier-etal-2025-findings</v>
+        <v/>
       </c>
       <c r="AH92" t="str">
         <f t="shared" si="26"/>
@@ -19312,11 +19294,11 @@
       </c>
       <c r="AI92" t="str">
         <f t="shared" si="27"/>
-        <v/>
+        <v>chang2025globalpiqaevaluatingphysical</v>
       </c>
       <c r="AK92">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:37">
@@ -19326,13 +19308,16 @@
       </c>
       <c r="B93" t="str" cm="1">
         <f t="array" ref="B93">_xlfn.IFS(ISBLANK(D93),"",ISBLANK(C93),"no venue",ISBLANK(E93),"no bib",ISNUMBER(SEARCH("xiv", C93)),"arxiv",SUM(I93:AA93)&lt;3,"no categories",TRUE,"")</f>
-        <v>no bib</v>
-      </c>
-      <c r="C93" t="s">
-        <v>342</v>
+        <v/>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>308</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
+      </c>
+      <c r="E93" s="12" t="s">
+        <v>352</v>
       </c>
       <c r="G93">
         <v>2026</v>
@@ -19343,28 +19328,37 @@
       <c r="I93">
         <v>1</v>
       </c>
-      <c r="L93">
-        <v>1</v>
-      </c>
       <c r="N93">
         <v>1</v>
       </c>
-      <c r="P93">
+      <c r="O93">
         <v>1</v>
       </c>
       <c r="Q93">
         <v>1</v>
       </c>
+      <c r="R93">
+        <v>1</v>
+      </c>
       <c r="S93">
         <v>1</v>
       </c>
-      <c r="Y93">
+      <c r="T93">
+        <v>1</v>
+      </c>
+      <c r="U93">
+        <v>1</v>
+      </c>
+      <c r="V93">
         <v>1</v>
       </c>
       <c r="Z93">
         <v>1</v>
       </c>
       <c r="AA93">
+        <v>1</v>
+      </c>
+      <c r="AB93">
         <v>1</v>
       </c>
       <c r="AD93">
@@ -19374,21 +19368,21 @@
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
-      <c r="AG93">
+      <c r="AG93" t="str">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>charpentier-etal-2025-findings</v>
       </c>
       <c r="AH93" t="str">
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="AI93">
+      <c r="AI93" t="str">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AK93">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:37">
@@ -19398,16 +19392,13 @@
       </c>
       <c r="B94" t="str" cm="1">
         <f t="array" ref="B94">_xlfn.IFS(ISBLANK(D94),"",ISBLANK(C94),"no venue",ISBLANK(E94),"no bib",ISNUMBER(SEARCH("xiv", C94)),"arxiv",SUM(I94:AA94)&lt;3,"no categories",TRUE,"")</f>
-        <v>arxiv</v>
+        <v>no bib</v>
       </c>
       <c r="C94" t="s">
-        <v>342</v>
-      </c>
-      <c r="D94" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="E94" s="12" t="s">
-        <v>357</v>
+        <v>340</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>354</v>
       </c>
       <c r="G94">
         <v>2026</v>
@@ -19415,22 +19406,28 @@
       <c r="H94">
         <v>1</v>
       </c>
-      <c r="O94">
-        <v>1</v>
-      </c>
-      <c r="R94">
+      <c r="I94">
+        <v>1</v>
+      </c>
+      <c r="L94">
+        <v>1</v>
+      </c>
+      <c r="N94">
+        <v>1</v>
+      </c>
+      <c r="P94">
+        <v>1</v>
+      </c>
+      <c r="Q94">
         <v>1</v>
       </c>
       <c r="S94">
         <v>1</v>
       </c>
-      <c r="U94">
-        <v>1</v>
-      </c>
-      <c r="W94">
-        <v>1</v>
-      </c>
       <c r="Y94">
+        <v>1</v>
+      </c>
+      <c r="Z94">
         <v>1</v>
       </c>
       <c r="AA94">
@@ -19441,19 +19438,19 @@
       </c>
       <c r="AF94">
         <f t="shared" si="24"/>
+        <v>1</v>
+      </c>
+      <c r="AG94">
+        <f t="shared" si="25"/>
         <v>0</v>
-      </c>
-      <c r="AG94" t="str">
-        <f t="shared" si="25"/>
-        <v/>
       </c>
       <c r="AH94" t="str">
         <f t="shared" si="26"/>
-        <v>suarez2026commonlid</v>
-      </c>
-      <c r="AI94" t="str">
+        <v/>
+      </c>
+      <c r="AI94">
         <f t="shared" si="27"/>
-        <v>suarez2026commonlid</v>
+        <v>0</v>
       </c>
       <c r="AK94">
         <f t="shared" si="28"/>
@@ -19470,13 +19467,13 @@
         <v>arxiv</v>
       </c>
       <c r="C95" t="s">
-        <v>342</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>359</v>
+        <v>340</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>356</v>
       </c>
       <c r="E95" s="12" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="G95">
         <v>2026</v>
@@ -19484,25 +19481,22 @@
       <c r="H95">
         <v>1</v>
       </c>
-      <c r="K95">
-        <v>1</v>
-      </c>
-      <c r="P95">
-        <v>1</v>
-      </c>
-      <c r="Q95">
+      <c r="O95">
+        <v>1</v>
+      </c>
+      <c r="R95">
         <v>1</v>
       </c>
       <c r="S95">
         <v>1</v>
       </c>
+      <c r="U95">
+        <v>1</v>
+      </c>
       <c r="W95">
         <v>1</v>
       </c>
       <c r="Y95">
-        <v>1</v>
-      </c>
-      <c r="Z95">
         <v>1</v>
       </c>
       <c r="AA95">
@@ -19513,19 +19507,19 @@
       </c>
       <c r="AF95">
         <f t="shared" si="24"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG95" t="str">
         <f t="shared" si="25"/>
-        <v>rahamim2026will</v>
+        <v/>
       </c>
       <c r="AH95" t="str">
         <f t="shared" si="26"/>
-        <v>rahamim2026will</v>
+        <v>suarez2026commonlid</v>
       </c>
       <c r="AI95" t="str">
         <f t="shared" si="27"/>
-        <v>rahamim2026will</v>
+        <v>suarez2026commonlid</v>
       </c>
       <c r="AK95">
         <f t="shared" si="28"/>
@@ -19542,13 +19536,13 @@
         <v>arxiv</v>
       </c>
       <c r="C96" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="E96" s="12" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="G96">
         <v>2026</v>
@@ -19556,13 +19550,25 @@
       <c r="H96">
         <v>1</v>
       </c>
-      <c r="O96">
+      <c r="K96">
+        <v>1</v>
+      </c>
+      <c r="P96">
         <v>1</v>
       </c>
       <c r="Q96">
         <v>1</v>
       </c>
-      <c r="T96">
+      <c r="S96">
+        <v>1</v>
+      </c>
+      <c r="W96">
+        <v>1</v>
+      </c>
+      <c r="Y96">
+        <v>1</v>
+      </c>
+      <c r="Z96">
         <v>1</v>
       </c>
       <c r="AA96">
@@ -19577,15 +19583,15 @@
       </c>
       <c r="AG96" t="str">
         <f t="shared" si="25"/>
-        <v>ashury2026errormap</v>
+        <v>rahamim2026will</v>
       </c>
       <c r="AH96" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>rahamim2026will</v>
       </c>
       <c r="AI96" t="str">
         <f t="shared" si="27"/>
-        <v/>
+        <v>rahamim2026will</v>
       </c>
       <c r="AK96">
         <f t="shared" si="28"/>
@@ -19602,13 +19608,13 @@
         <v>arxiv</v>
       </c>
       <c r="C97" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D97" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="E97" s="12" t="s">
         <v>362</v>
-      </c>
-      <c r="E97" s="12" t="s">
-        <v>363</v>
       </c>
       <c r="G97">
         <v>2026</v>
@@ -19619,13 +19625,10 @@
       <c r="O97">
         <v>1</v>
       </c>
-      <c r="P97">
+      <c r="Q97">
         <v>1</v>
       </c>
       <c r="T97">
-        <v>1</v>
-      </c>
-      <c r="X97">
         <v>1</v>
       </c>
       <c r="AA97">
@@ -19640,7 +19643,7 @@
       </c>
       <c r="AG97" t="str">
         <f t="shared" si="25"/>
-        <v>ashury2026robustness</v>
+        <v>ashury2026errormap</v>
       </c>
       <c r="AH97" t="str">
         <f t="shared" si="26"/>
@@ -19661,35 +19664,56 @@
         <v>97</v>
       </c>
       <c r="B98" t="str" cm="1">
-        <f t="array" ref="B98">_xlfn.IFS(ISBLANK(D99),"",ISBLANK(C98),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C98)),"arxiv",SUM(I98:AA98)&lt;3,"no categories",TRUE,"")</f>
+        <f t="array" ref="B98">_xlfn.IFS(ISBLANK(D98),"",ISBLANK(C98),"no venue",ISBLANK(E98),"no bib",ISNUMBER(SEARCH("xiv", C98)),"arxiv",SUM(I98:AA98)&lt;3,"no categories",TRUE,"")</f>
         <v>arxiv</v>
       </c>
       <c r="C98" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="E98" s="12" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="G98">
         <v>2026</v>
       </c>
+      <c r="H98">
+        <v>1</v>
+      </c>
+      <c r="O98">
+        <v>1</v>
+      </c>
+      <c r="P98">
+        <v>1</v>
+      </c>
+      <c r="T98">
+        <v>1</v>
+      </c>
+      <c r="X98">
+        <v>1</v>
+      </c>
+      <c r="AA98">
+        <v>1</v>
+      </c>
+      <c r="AD98">
+        <v>1</v>
+      </c>
       <c r="AF98">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG98" t="str">
-        <f>IF(AF98,#REF!,"")</f>
+        <f t="shared" si="25"/>
+        <v>ashury2026robustness</v>
+      </c>
+      <c r="AH98" t="str">
+        <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="AH98" t="str">
-        <f>IF(W98,#REF!,"")</f>
-        <v/>
-      </c>
       <c r="AI98" t="str">
-        <f>IF(Y98,#REF!,"")</f>
+        <f t="shared" si="27"/>
         <v/>
       </c>
       <c r="AK98">
@@ -19697,62 +19721,207 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:37" ht="17">
+    <row r="99" spans="1:37">
       <c r="A99">
         <f t="shared" si="23"/>
         <v>98</v>
       </c>
       <c r="B99" t="str" cm="1">
-        <f t="array" ref="B99">_xlfn.IFS(ISBLANK(#REF!),"",ISBLANK(C99),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C99)),"arxiv",SUM(I99:AA99)&lt;3,"no categories",TRUE,"")</f>
+        <f t="array" ref="B99">_xlfn.IFS(ISBLANK(D100),"",ISBLANK(C99),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C99)),"arxiv",SUM(I99:AA99)&lt;3,"no categories",TRUE,"")</f>
         <v>arxiv</v>
       </c>
       <c r="C99" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D99" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="E99" s="12" t="s">
         <v>368</v>
-      </c>
-      <c r="E99" s="12" t="s">
-        <v>371</v>
       </c>
       <c r="G99">
         <v>2026</v>
       </c>
-      <c r="AG99" s="8"/>
+      <c r="H99">
+        <v>1</v>
+      </c>
+      <c r="K99">
+        <v>1</v>
+      </c>
+      <c r="P99">
+        <v>1</v>
+      </c>
+      <c r="T99">
+        <v>1</v>
+      </c>
+      <c r="U99">
+        <v>1</v>
+      </c>
+      <c r="W99">
+        <v>1</v>
+      </c>
+      <c r="X99">
+        <v>1</v>
+      </c>
+      <c r="AA99">
+        <v>1</v>
+      </c>
+      <c r="AD99">
+        <v>1</v>
+      </c>
+      <c r="AF99">
+        <f t="shared" si="24"/>
+        <v>1</v>
+      </c>
+      <c r="AG99" t="e">
+        <f>IF(AF99,#REF!,"")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AH99" t="e">
+        <f>IF(W99,#REF!,"")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AI99" t="str">
+        <f>IF(Y99,#REF!,"")</f>
+        <v/>
+      </c>
+      <c r="AK99">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="100" spans="1:37" ht="35">
+    <row r="100" spans="1:37" ht="17">
       <c r="A100">
         <f t="shared" si="23"/>
         <v>99</v>
       </c>
       <c r="B100" t="str" cm="1">
-        <f t="array" ref="B100">_xlfn.IFS(ISBLANK(D100),"",ISBLANK(C100),"no venue",ISBLANK(E100),"no bib",ISNUMBER(SEARCH("xiv", C100)),"arxiv",SUM(I100:AA100)&lt;3,"no categories",TRUE,"")</f>
+        <f t="array" ref="B100">_xlfn.IFS(ISBLANK(#REF!),"",ISBLANK(C100),"no venue",ISBLANK(#REF!),"no bib",ISNUMBER(SEARCH("xiv", C100)),"arxiv",SUM(I100:AA100)&lt;3,"no categories",TRUE,"")</f>
         <v>arxiv</v>
       </c>
       <c r="C100" t="s">
-        <v>342</v>
-      </c>
-      <c r="D100" s="16" t="s">
-        <v>372</v>
+        <v>340</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>366</v>
       </c>
       <c r="E100" s="12" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="G100">
         <v>2026</v>
       </c>
+      <c r="H100">
+        <v>1</v>
+      </c>
+      <c r="N100">
+        <v>1</v>
+      </c>
+      <c r="O100">
+        <v>1</v>
+      </c>
+      <c r="Q100">
+        <v>1</v>
+      </c>
+      <c r="R100">
+        <v>1</v>
+      </c>
+      <c r="T100">
+        <v>1</v>
+      </c>
+      <c r="W100">
+        <v>1</v>
+      </c>
+      <c r="X100">
+        <v>1</v>
+      </c>
+      <c r="Y100">
+        <v>1</v>
+      </c>
+      <c r="AA100">
+        <v>1</v>
+      </c>
+      <c r="AD100">
+        <v>1</v>
+      </c>
       <c r="AG100" s="8"/>
+      <c r="AH100" t="e">
+        <f>IF(W100,#REF!,"")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AK100">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="101" spans="1:37" ht="17">
+    <row r="101" spans="1:37" ht="35">
       <c r="A101">
         <f t="shared" si="23"/>
         <v>100</v>
       </c>
       <c r="B101" t="str" cm="1">
         <f t="array" ref="B101">_xlfn.IFS(ISBLANK(D101),"",ISBLANK(C101),"no venue",ISBLANK(E101),"no bib",ISNUMBER(SEARCH("xiv", C101)),"arxiv",SUM(I101:AA101)&lt;3,"no categories",TRUE,"")</f>
-        <v/>
+        <v>arxiv</v>
+      </c>
+      <c r="C101" t="s">
+        <v>340</v>
+      </c>
+      <c r="D101" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="E101" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="G101">
+        <v>2026</v>
+      </c>
+      <c r="H101">
+        <v>1</v>
+      </c>
+      <c r="O101">
+        <v>1</v>
+      </c>
+      <c r="Q101">
+        <v>1</v>
+      </c>
+      <c r="R101">
+        <v>1</v>
+      </c>
+      <c r="S101">
+        <v>1</v>
+      </c>
+      <c r="T101">
+        <v>1</v>
+      </c>
+      <c r="U101">
+        <v>1</v>
+      </c>
+      <c r="W101">
+        <v>1</v>
+      </c>
+      <c r="X101">
+        <v>1</v>
+      </c>
+      <c r="Y101">
+        <v>1</v>
+      </c>
+      <c r="Z101">
+        <v>1</v>
+      </c>
+      <c r="AA101">
+        <v>1</v>
+      </c>
+      <c r="AC101">
+        <v>1</v>
+      </c>
+      <c r="AD101">
+        <v>1</v>
       </c>
       <c r="AG101" s="8"/>
+      <c r="AK101">
+        <f t="shared" si="28"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="102" spans="1:37" ht="17">
       <c r="A102">
@@ -20041,6 +20210,14 @@
       <c r="AG127" s="8"/>
     </row>
     <row r="128" spans="1:33" ht="17">
+      <c r="A128">
+        <f t="shared" si="23"/>
+        <v>127</v>
+      </c>
+      <c r="B128" t="str" cm="1">
+        <f t="array" ref="B128">_xlfn.IFS(ISBLANK(D128),"",ISBLANK(C128),"no venue",ISBLANK(E128),"no bib",ISNUMBER(SEARCH("xiv", C128)),"arxiv",SUM(I128:AA128)&lt;3,"no categories",TRUE,"")</f>
+        <v/>
+      </c>
       <c r="AG128" s="8"/>
     </row>
     <row r="129" spans="7:36" ht="17">
@@ -20064,229 +20241,232 @@
     <row r="135" spans="7:36" ht="17">
       <c r="AG135" s="8"/>
     </row>
-    <row r="137" spans="7:36">
-      <c r="G137" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H137">
-        <f>SUM(H2:H79)</f>
-        <v>77</v>
-      </c>
-      <c r="I137">
-        <f t="shared" ref="I137:N137" si="30">SUM(I2:I78)</f>
-        <v>6</v>
-      </c>
-      <c r="J137">
-        <f t="shared" si="30"/>
-        <v>5</v>
-      </c>
-      <c r="K137">
-        <f t="shared" si="30"/>
-        <v>11</v>
-      </c>
-      <c r="L137">
-        <f t="shared" si="30"/>
-        <v>2</v>
-      </c>
-      <c r="M137">
-        <f t="shared" si="30"/>
-        <v>4</v>
-      </c>
-      <c r="N137">
-        <f t="shared" si="30"/>
-        <v>4</v>
-      </c>
-      <c r="O137">
-        <f>SUM(O2:O79)</f>
-        <v>39</v>
-      </c>
-      <c r="P137">
-        <f>SUM(P2:P78)</f>
-        <v>42</v>
-      </c>
-      <c r="Q137">
-        <f>SUM(Q2:Q78)</f>
-        <v>43</v>
-      </c>
-      <c r="R137">
-        <f>SUM(R2:R78)</f>
-        <v>21</v>
-      </c>
-      <c r="S137">
-        <f>SUM(S2:S78)</f>
-        <v>32</v>
-      </c>
-      <c r="T137">
-        <f>SUM(T2:T79)</f>
-        <v>40</v>
-      </c>
-      <c r="U137">
-        <f>SUM(U2:U78)</f>
-        <v>15</v>
-      </c>
-      <c r="V137">
-        <f>SUM(V2:V78)</f>
-        <v>31</v>
-      </c>
-      <c r="W137">
-        <f>SUM(W2:W79)</f>
-        <v>33</v>
-      </c>
-      <c r="X137">
-        <f>SUM(X2:X78)</f>
-        <v>35</v>
-      </c>
-      <c r="Y137">
-        <f>SUM(Y2:Y79)</f>
-        <v>35</v>
-      </c>
-      <c r="Z137">
-        <f>SUM(Z2:Z78)</f>
-        <v>40</v>
-      </c>
-      <c r="AA137">
-        <f>SUM(AA2:AA78)</f>
-        <v>74</v>
-      </c>
-      <c r="AD137">
-        <f>COUNT(A2:A78)</f>
-        <v>77</v>
-      </c>
-      <c r="AE137">
-        <f>SUM(AE2:AE79)</f>
-        <v>7</v>
-      </c>
-      <c r="AF137">
-        <f>SUM(AF2:AF79)</f>
-        <v>63</v>
-      </c>
-      <c r="AG137" t="str">
-        <f>IF(AF137,E80,"")</f>
-        <v>ashurytahan2025mightytorrbenchmarktable</v>
-      </c>
-      <c r="AH137" t="str">
-        <f>IF(W137,E80,"")</f>
-        <v>ashurytahan2025mightytorrbenchmarktable</v>
-      </c>
-      <c r="AI137" t="str">
-        <f>IF(Y137,E80,"")</f>
-        <v>ashurytahan2025mightytorrbenchmarktable</v>
-      </c>
-      <c r="AJ137" t="str">
-        <f>IF(AE137,E80,"")</f>
-        <v>ashurytahan2025mightytorrbenchmarktable</v>
-      </c>
+    <row r="136" spans="7:36" ht="17">
+      <c r="AG136" s="8"/>
     </row>
     <row r="138" spans="7:36">
       <c r="G138" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H138" s="7">
-        <f t="shared" ref="H138:AA138" si="31">H137/$AD$137</f>
-        <v>1</v>
-      </c>
-      <c r="I138" s="7">
-        <f t="shared" si="31"/>
+        <v>178</v>
+      </c>
+      <c r="H138">
+        <f>SUM(H2:H79)</f>
+        <v>77</v>
+      </c>
+      <c r="I138">
+        <f t="shared" ref="I138:N138" si="35">SUM(I2:I78)</f>
+        <v>6</v>
+      </c>
+      <c r="J138">
+        <f t="shared" si="35"/>
+        <v>5</v>
+      </c>
+      <c r="K138">
+        <f t="shared" si="35"/>
+        <v>11</v>
+      </c>
+      <c r="L138">
+        <f t="shared" si="35"/>
+        <v>2</v>
+      </c>
+      <c r="M138">
+        <f t="shared" si="35"/>
+        <v>4</v>
+      </c>
+      <c r="N138">
+        <f t="shared" si="35"/>
+        <v>5</v>
+      </c>
+      <c r="O138">
+        <f>SUM(O2:O79)</f>
+        <v>39</v>
+      </c>
+      <c r="P138">
+        <f>SUM(P2:P78)</f>
+        <v>42</v>
+      </c>
+      <c r="Q138">
+        <f>SUM(Q2:Q78)</f>
+        <v>43</v>
+      </c>
+      <c r="R138">
+        <f>SUM(R2:R78)</f>
+        <v>21</v>
+      </c>
+      <c r="S138">
+        <f>SUM(S2:S78)</f>
+        <v>32</v>
+      </c>
+      <c r="T138">
+        <f>SUM(T2:T79)</f>
+        <v>40</v>
+      </c>
+      <c r="U138">
+        <f>SUM(U2:U78)</f>
+        <v>15</v>
+      </c>
+      <c r="V138">
+        <f>SUM(V2:V78)</f>
+        <v>31</v>
+      </c>
+      <c r="W138">
+        <f>SUM(W2:W79)</f>
+        <v>33</v>
+      </c>
+      <c r="X138">
+        <f>SUM(X2:X78)</f>
+        <v>35</v>
+      </c>
+      <c r="Y138">
+        <f>SUM(Y2:Y79)</f>
+        <v>35</v>
+      </c>
+      <c r="Z138">
+        <f>SUM(Z2:Z78)</f>
+        <v>40</v>
+      </c>
+      <c r="AA138">
+        <f>SUM(AA2:AA78)</f>
+        <v>74</v>
+      </c>
+      <c r="AD138">
+        <f>COUNT(A2:A78)</f>
+        <v>77</v>
+      </c>
+      <c r="AE138">
+        <f>SUM(AE2:AE79)</f>
+        <v>7</v>
+      </c>
+      <c r="AF138">
+        <f>SUM(AF2:AF79)</f>
+        <v>63</v>
+      </c>
+      <c r="AG138" t="str">
+        <f>IF(AF138,E80,"")</f>
+        <v>ashurytahan2025mightytorrbenchmarktable</v>
+      </c>
+      <c r="AH138" t="str">
+        <f>IF(W138,E80,"")</f>
+        <v>ashurytahan2025mightytorrbenchmarktable</v>
+      </c>
+      <c r="AI138" t="str">
+        <f>IF(Y138,E80,"")</f>
+        <v>ashurytahan2025mightytorrbenchmarktable</v>
+      </c>
+      <c r="AJ138" t="str">
+        <f>IF(AE138,E80,"")</f>
+        <v>ashurytahan2025mightytorrbenchmarktable</v>
+      </c>
+    </row>
+    <row r="139" spans="7:36">
+      <c r="G139" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="H139" s="7">
+        <f t="shared" ref="H139:AA139" si="36">H138/$AD$138</f>
+        <v>1</v>
+      </c>
+      <c r="I139" s="7">
+        <f t="shared" si="36"/>
         <v>7.792207792207792E-2</v>
       </c>
-      <c r="J138" s="7">
-        <f t="shared" si="31"/>
+      <c r="J139" s="7">
+        <f t="shared" si="36"/>
         <v>6.4935064935064929E-2</v>
       </c>
-      <c r="K138" s="7">
-        <f t="shared" si="31"/>
+      <c r="K139" s="7">
+        <f t="shared" si="36"/>
         <v>0.14285714285714285</v>
       </c>
-      <c r="L138" s="7">
-        <f t="shared" si="31"/>
+      <c r="L139" s="7">
+        <f t="shared" si="36"/>
         <v>2.5974025974025976E-2</v>
       </c>
-      <c r="M138" s="7">
-        <f t="shared" si="31"/>
+      <c r="M139" s="7">
+        <f t="shared" si="36"/>
         <v>5.1948051948051951E-2</v>
       </c>
-      <c r="N138" s="7">
-        <f t="shared" si="31"/>
-        <v>5.1948051948051951E-2</v>
-      </c>
-      <c r="O138" s="7">
-        <f t="shared" si="31"/>
+      <c r="N139" s="7">
+        <f t="shared" si="36"/>
+        <v>6.4935064935064929E-2</v>
+      </c>
+      <c r="O139" s="7">
+        <f t="shared" si="36"/>
         <v>0.50649350649350644</v>
       </c>
-      <c r="P138" s="7">
-        <f t="shared" si="31"/>
+      <c r="P139" s="7">
+        <f t="shared" si="36"/>
         <v>0.54545454545454541</v>
       </c>
-      <c r="Q138" s="7">
-        <f t="shared" si="31"/>
+      <c r="Q139" s="7">
+        <f t="shared" si="36"/>
         <v>0.55844155844155841</v>
       </c>
-      <c r="R138" s="7">
-        <f t="shared" si="31"/>
+      <c r="R139" s="7">
+        <f t="shared" si="36"/>
         <v>0.27272727272727271</v>
       </c>
-      <c r="S138" s="7">
-        <f t="shared" si="31"/>
+      <c r="S139" s="7">
+        <f t="shared" si="36"/>
         <v>0.41558441558441561</v>
       </c>
-      <c r="T138" s="7">
-        <f t="shared" si="31"/>
+      <c r="T139" s="7">
+        <f t="shared" si="36"/>
         <v>0.51948051948051943</v>
       </c>
-      <c r="U138" s="7">
-        <f t="shared" si="31"/>
+      <c r="U139" s="7">
+        <f t="shared" si="36"/>
         <v>0.19480519480519481</v>
       </c>
-      <c r="V138" s="7">
-        <f t="shared" si="31"/>
+      <c r="V139" s="7">
+        <f t="shared" si="36"/>
         <v>0.40259740259740262</v>
       </c>
-      <c r="W138" s="7">
-        <f t="shared" si="31"/>
+      <c r="W139" s="7">
+        <f t="shared" si="36"/>
         <v>0.42857142857142855</v>
       </c>
-      <c r="X138" s="7">
-        <f t="shared" si="31"/>
+      <c r="X139" s="7">
+        <f t="shared" si="36"/>
         <v>0.45454545454545453</v>
       </c>
-      <c r="Y138" s="7">
-        <f t="shared" si="31"/>
+      <c r="Y139" s="7">
+        <f t="shared" si="36"/>
         <v>0.45454545454545453</v>
       </c>
-      <c r="Z138" s="7">
-        <f t="shared" si="31"/>
+      <c r="Z139" s="7">
+        <f t="shared" si="36"/>
         <v>0.51948051948051943</v>
       </c>
-      <c r="AA138" s="7">
-        <f t="shared" si="31"/>
+      <c r="AA139" s="7">
+        <f t="shared" si="36"/>
         <v>0.96103896103896103</v>
       </c>
-      <c r="AB138" s="7"/>
-      <c r="AC138" s="7"/>
-      <c r="AD138">
+      <c r="AB139" s="7"/>
+      <c r="AC139" s="7"/>
+      <c r="AD139">
         <f>COUNT(A3:A80)</f>
         <v>78</v>
       </c>
-      <c r="AG138" t="str">
-        <f>IF(AF138,#REF!,"")</f>
+      <c r="AG139" t="str">
+        <f>IF(AF139,#REF!,"")</f>
         <v/>
       </c>
-      <c r="AH138" t="e">
-        <f>IF(W138,#REF!,"")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AI138" t="e">
-        <f>IF(Y138,#REF!,"")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AJ138" t="str">
-        <f>IF(AE138,#REF!,"")</f>
+      <c r="AH139" t="e">
+        <f>IF(W139,#REF!,"")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AI139" t="e">
+        <f>IF(Y139,#REF!,"")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AJ139" t="str">
+        <f>IF(AE139,#REF!,"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AK78" xr:uid="{92277768-849A-7540-AC05-5E1BE041CC8E}"/>
-  <conditionalFormatting sqref="B2:B127">
+  <conditionalFormatting sqref="B2:B128">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -20342,16 +20522,17 @@
     <hyperlink ref="D87" r:id="rId41" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:cFHS6HbyZ2cC" xr:uid="{012D4D4B-F7DB-534F-929E-F3980EB01887}"/>
     <hyperlink ref="D89" r:id="rId42" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:OU6Ihb5iCvQC" xr:uid="{83F89CA5-9C53-454A-82C0-5B114240419E}"/>
     <hyperlink ref="D88" r:id="rId43" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:p2g8aNsByqUC" xr:uid="{F1C14A89-89CC-4F40-8425-EE9E1FA18475}"/>
-    <hyperlink ref="D90" r:id="rId44" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:738O_yMBCRsC" xr:uid="{7F06036E-46CB-7B4A-B5A9-01BD9FEB494D}"/>
-    <hyperlink ref="D91" r:id="rId45" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:K3LRdlH-MEoC" xr:uid="{E3BF1F50-9A61-BD47-80DD-3E7FA5F51488}"/>
-    <hyperlink ref="D92" r:id="rId46" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:tOudhMTPpwUC" xr:uid="{A1EF67F5-E28E-A14D-A57D-7545932AF158}"/>
-    <hyperlink ref="C92" r:id="rId47" display="BabyLM@EMNLP" xr:uid="{D8DDEF9E-B21E-CD40-A406-DFC0EB019B6A}"/>
-    <hyperlink ref="D93" r:id="rId48" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:4fKUyHm3Qg0C" xr:uid="{63AC3719-785D-4045-842F-51673617DEA4}"/>
-    <hyperlink ref="D95" r:id="rId49" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:B3FOqHPlNUQC" xr:uid="{4655ADB8-FEB9-6148-99F7-03736D7EB3B9}"/>
-    <hyperlink ref="D96" r:id="rId50" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:sSrBHYA8nusC" xr:uid="{94FB61E5-5F04-5645-A99F-119289B9E81D}"/>
-    <hyperlink ref="D97" r:id="rId51" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:5Ul4iDaHHb8C" xr:uid="{AC018292-7C41-B947-89FB-2E8002093149}"/>
-    <hyperlink ref="D99" r:id="rId52" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:eflP2zaiRacC" xr:uid="{60D0073E-0896-9C4A-A723-621180E109EC}"/>
-    <hyperlink ref="D98" r:id="rId53" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:VOx2b1Wkg3QC" xr:uid="{1B316D5B-F142-5C4C-8594-5D8D28179250}"/>
+    <hyperlink ref="D91" r:id="rId44" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:738O_yMBCRsC" xr:uid="{7F06036E-46CB-7B4A-B5A9-01BD9FEB494D}"/>
+    <hyperlink ref="D92" r:id="rId45" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:K3LRdlH-MEoC" xr:uid="{E3BF1F50-9A61-BD47-80DD-3E7FA5F51488}"/>
+    <hyperlink ref="D93" r:id="rId46" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:tOudhMTPpwUC" xr:uid="{A1EF67F5-E28E-A14D-A57D-7545932AF158}"/>
+    <hyperlink ref="C93" r:id="rId47" display="BabyLM@EMNLP" xr:uid="{D8DDEF9E-B21E-CD40-A406-DFC0EB019B6A}"/>
+    <hyperlink ref="D94" r:id="rId48" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:4fKUyHm3Qg0C" xr:uid="{63AC3719-785D-4045-842F-51673617DEA4}"/>
+    <hyperlink ref="D96" r:id="rId49" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:B3FOqHPlNUQC" xr:uid="{4655ADB8-FEB9-6148-99F7-03736D7EB3B9}"/>
+    <hyperlink ref="D97" r:id="rId50" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:sSrBHYA8nusC" xr:uid="{94FB61E5-5F04-5645-A99F-119289B9E81D}"/>
+    <hyperlink ref="D98" r:id="rId51" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:5Ul4iDaHHb8C" xr:uid="{AC018292-7C41-B947-89FB-2E8002093149}"/>
+    <hyperlink ref="D100" r:id="rId52" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:eflP2zaiRacC" xr:uid="{60D0073E-0896-9C4A-A723-621180E109EC}"/>
+    <hyperlink ref="D99" r:id="rId53" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:VOx2b1Wkg3QC" xr:uid="{1B316D5B-F142-5C4C-8594-5D8D28179250}"/>
+    <hyperlink ref="D63" r:id="rId54" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=8b8IhUYAAAAJ&amp;cstart=20&amp;pagesize=80&amp;sortby=pubdate&amp;citation_for_view=8b8IhUYAAAAJ:uWQEDVKXjbEC" xr:uid="{7F1AF470-D2BE-F040-AB43-BAACD4F06829}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -24574,7 +24755,7 @@
       </c>
       <c r="C61" t="str">
         <f>Sheet1!D63</f>
-        <v xml:space="preserve"> Learning from Naturally Occurring Feedback</v>
+        <v>Naturally occurring feedback is common, extractable and useful</v>
       </c>
       <c r="D61" t="str">
         <f>Sheet1!F63</f>
@@ -29625,7 +29806,7 @@
       </c>
       <c r="C61" t="str">
         <f>Sheet1!D63</f>
-        <v xml:space="preserve"> Learning from Naturally Occurring Feedback</v>
+        <v>Naturally occurring feedback is common, extractable and useful</v>
       </c>
       <c r="D61" t="str">
         <f>Sheet1!F63</f>

</xml_diff>

<commit_message>
Harden and consolidate the publications pipeline
- update.py: mtime-based auto-skip for all 4 steps; step 4 calls
  publications.main() directly (no subprocess); --force/--fetch-age flags
- update.py step 2: show closest xlsx match for each flagged new paper
- resolve_arxiv.py: DBLP title validation (0.72 similarity threshold);
  dedup guard before bib append; CRLF regex fix
- fetch_citations.py: atomic CSV write; raise on 0-paper fetch
- publications.py: consolidate parse_bibtex from augment_bib; remove numpy
- augment_bib.py: remove dead code (enhanced.bib generator, unused helpers)
- .gitignore: added

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contributions_table.xlsx
+++ b/Contributions_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lc/PycharmProjects/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B85019C-85BF-0946-A90F-470EED35ACAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91506202-1311-DE49-B8E5-89AC03A88D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{5AA491FB-7947-2140-ACD9-201A623594D0}"/>
   </bookViews>
@@ -14023,7 +14023,7 @@
         <v>89</v>
       </c>
       <c r="G22">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -14088,7 +14088,7 @@
         <v>87</v>
       </c>
       <c r="G23">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -22290,7 +22290,7 @@
       </c>
       <c r="E22">
         <f>Sheet1!G22</f>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F22" t="e">
         <f>F23+Sheet1!O22</f>
@@ -22360,7 +22360,7 @@
       </c>
       <c r="E23">
         <f>Sheet1!G23</f>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F23" t="e">
         <f>F24+Sheet1!O23</f>
@@ -27341,7 +27341,7 @@
       </c>
       <c r="E22">
         <f>Sheet1!G22</f>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F22" t="e">
         <f>Commulative!F22/Commulative!$A22</f>
@@ -27411,7 +27411,7 @@
       </c>
       <c r="E23">
         <f>Sheet1!G23</f>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F23" t="e">
         <f>Commulative!F23/Commulative!$A23</f>

</xml_diff>